<commit_message>
Implement Q1 second revision: official M1, curtailment bound, and sensitivity.
Lock attachment row order, parameterize the LP, and export baseline plus PCC cases without overwriting the official plan.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/output/result1.xlsx
+++ b/output/result1.xlsx
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>1.893918988571386e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" ht="14" customHeight="1">
@@ -1134,7 +1134,7 @@
         </is>
       </c>
       <c r="B68" s="7" t="n">
-        <v>415.1176493268283</v>
+        <v>415.1176703703735</v>
       </c>
     </row>
     <row r="69" ht="14" customHeight="1">
@@ -1554,7 +1554,7 @@
         </is>
       </c>
       <c r="B110" s="7" t="n">
-        <v>64.53438871506815</v>
+        <v>64.53438871506819</v>
       </c>
     </row>
     <row r="111" ht="14" customHeight="1">
@@ -1984,7 +1984,7 @@
         <v>833.3333333333333</v>
       </c>
       <c r="C3" t="n">
-        <v>6956.98138106081</v>
+        <v>6956.9814</v>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
@@ -2002,7 +2002,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4448.633849326828</v>
+        <v>4448.633870370373</v>
       </c>
       <c r="C4" t="n">
         <v>1702.996983333333</v>

</xml_diff>